<commit_message>
Changes of quiz and scorm
</commit_message>
<xml_diff>
--- a/public/sample/QuizSection.xlsx
+++ b/public/sample/QuizSection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pc\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA97E139-9733-4345-8258-B4AF32D49490}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B8F07FB-F305-4506-A7FF-244F8669B137}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,8 +19,114 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Pc</author>
+  </authors>
+  <commentList>
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{0D98963C-1F6D-4D2D-9D37-AD9D4AA1BB90}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Pc:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Correct answer should be in array</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{B6AD676F-E723-47A2-BE63-48277B7D631F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Pc:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+use 1 for easy, 2 for medium, 3 for difficult</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{CD9E1C7E-BD6B-41AE-A125-966D257C1DDB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Pc:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Only true or false allowed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{4414B398-0D49-4AAC-A3CB-144EBE4D784F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Pc:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Use only Single Correct or Multiple Correct</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="56">
   <si>
     <t>Sno</t>
   </si>
@@ -56,13 +162,145 @@
   </si>
   <si>
     <t>Difficulty Level</t>
+  </si>
+  <si>
+    <t>Which gas is most abundant in Earth’s atmosphere?</t>
+  </si>
+  <si>
+    <t>Oxygen</t>
+  </si>
+  <si>
+    <t>Nitrogen</t>
+  </si>
+  <si>
+    <t>Carbon Dioxide</t>
+  </si>
+  <si>
+    <t>Argon</t>
+  </si>
+  <si>
+    <t>Science</t>
+  </si>
+  <si>
+    <t>This is the medium question</t>
+  </si>
+  <si>
+    <t>Single Correct</t>
+  </si>
+  <si>
+    <t>Which of the following statements about DNA are true?</t>
+  </si>
+  <si>
+    <t>DNA is double-stranded</t>
+  </si>
+  <si>
+    <t>DNA contains uracil</t>
+  </si>
+  <si>
+    <t>DNA has a sugar-phosphate backbone</t>
+  </si>
+  <si>
+    <t>DNA replication is semiconservative</t>
+  </si>
+  <si>
+    <t>[2]</t>
+  </si>
+  <si>
+    <t>Multiple Correct</t>
+  </si>
+  <si>
+    <t>Which of the following numbers are prime?</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>57</t>
+  </si>
+  <si>
+    <t>[1, 3]</t>
+  </si>
+  <si>
+    <t>Math</t>
+  </si>
+  <si>
+    <t>Who is known as the Father of the Nation (India)?</t>
+  </si>
+  <si>
+    <t>Jawaharlal Nehru</t>
+  </si>
+  <si>
+    <t>Mahatma Gandhi</t>
+  </si>
+  <si>
+    <t>Subhas Chandra Bose</t>
+  </si>
+  <si>
+    <t>Sardar Patel</t>
+  </si>
+  <si>
+    <t>GK</t>
+  </si>
+  <si>
+    <t>In a certain code, TREE = 94. What is the value of LEAF?</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>[3]</t>
+  </si>
+  <si>
+    <t>Reasoning</t>
+  </si>
+  <si>
+    <t>Which of the following statements about hashing are true?</t>
+  </si>
+  <si>
+    <t>Hash collisions can occur</t>
+  </si>
+  <si>
+    <t>Perfect hashing guarantees no collisions</t>
+  </si>
+  <si>
+    <t>Chaining is a collision resolution method</t>
+  </si>
+  <si>
+    <t>Load factor = (size of table) / (number of elements)</t>
+  </si>
+  <si>
+    <t>[1, 2, 3]</t>
+  </si>
+  <si>
+    <t>Question Type</t>
+  </si>
+  <si>
+    <t>Use Answer Explanation</t>
+  </si>
+  <si>
+    <t>[1, 3,  4]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -78,13 +316,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color rgb="FF222222"/>
       <name val="Arial"/>
@@ -95,6 +326,19 @@
       <color rgb="FF222222"/>
       <name val="Arial"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -123,7 +367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -136,18 +380,21 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -422,25 +669,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.42578125" customWidth="1"/>
     <col min="2" max="2" width="48.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="22.5703125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="28.85546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="27.42578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="42.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="43.85546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="46.7109375" style="2" customWidth="1"/>
     <col min="7" max="7" width="18.85546875" style="2" customWidth="1"/>
     <col min="8" max="8" width="26.42578125" style="2" customWidth="1"/>
     <col min="9" max="9" width="25.42578125" customWidth="1"/>
     <col min="10" max="10" width="19" customWidth="1"/>
-    <col min="11" max="11" width="9.28515625" customWidth="1"/>
-    <col min="12" max="12" width="20.28515625" customWidth="1"/>
+    <col min="11" max="11" width="17.5703125" customWidth="1"/>
+    <col min="12" max="12" width="32" customWidth="1"/>
+    <col min="13" max="13" width="28" customWidth="1"/>
+    <col min="14" max="14" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:14">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -465,7 +714,7 @@
       <c r="H1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="J1" s="3" t="s">
@@ -477,38 +726,231 @@
       <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="M1" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>53</v>
+      </c>
     </row>
-    <row r="2" spans="1:12">
-      <c r="B2" s="6"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="10"/>
+    <row r="2" spans="1:14">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="M2" t="b">
+        <v>1</v>
+      </c>
+      <c r="N2" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="3" spans="1:12">
-      <c r="B3" s="6"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="I3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="11"/>
+    <row r="3" spans="1:14">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="J3">
+        <v>3</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="L3" s="8"/>
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N3" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="4" spans="1:12">
-      <c r="B4" s="6"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="I4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="11"/>
+    <row r="4" spans="1:14">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="L4" s="8"/>
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="30">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="M6" t="b">
+        <v>0</v>
+      </c>
+      <c r="N6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="30">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J7">
+        <v>3</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="M7" t="b">
+        <v>0</v>
+      </c>
+      <c r="N7" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>